<commit_message>
Raise the free-play cargo budget from 55 t to 120 t
Playtesting showed one large Living Quarters ate half the budget. A base for
six needs roughly 65-80 t; 120 t leaves room for a generous design.
Missions keep their own per-landing payloads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>55000</v>
+        <v>120000</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
@@ -792,13 +792,16 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Landed cargo for a full habitat. About half of one large cargo lander. Missions can set smaller budgets.</t>
+          <t>Landed cargo for a full habitat in free play: enough for a generous base (about 100 room cells with equipment). Raised from 55,000 on 22 Oct after playtesting. Missions set their own per-landing payloads.</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
           <t>cargo_budget_kg</t>
         </is>
+      </c>
+      <c r="F4" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="5">
@@ -8175,7 +8178,6 @@
       </c>
       <c r="U85" s="8" t="n"/>
     </row>
-    <row r="86"/>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add resupply landers, the regolith printer and Mars-made material
- Survival starts with 80 t and gets +15 t every 3 sols; Freedom 120 t, +20 t every 2 sols
- Resupply landers land near the crew lander, stay as landmarks, and are saved
- Regolith printer (Storage/Engineering) and regolith intake (outdoors), new Blender models
- Mars-made material pays first for printable things: room shells, corridors, partitions, shelving, crates
- Cargo panel shows both pools; HUD counts down to the next resupply; printer arrives in Mission 6
- One SITE_MACHINES list replaces scattered solar/reactor/ice-drill checks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Landed cargo for a full habitat in free play: enough for a generous base (about 100 room cells with equipment). Raised from 55,000 on 22 Oct after playtesting. Missions set their own per-landing payloads.</t>
+          <t>Survival starting cargo. Lowered to 80,000 on 22 Oct: resupply landers and the regolith printer now grow the base over time. Freedom starts with more (below). Missions set their own per-landing payloads.</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1426,6 +1426,173 @@
       <c r="E29" s="10" t="inlineStr">
         <is>
           <t>danger_cold_c</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Freedom starting cargo</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Freedom: a generous start and bigger, quicker resupplies.</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>freedom_cargo_budget_kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Resupply interval (Survival)</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>sols</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>A resupply lander arrives this often. Real launch windows are about 26 months apart; the game compresses time.</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>resupply_sols_survival</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Resupply size (Survival)</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Cargo each Survival resupply lander brings.</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>resupply_kg_survival</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Resupply interval (Freedom)</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>sols</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>resupply_sols_freedom</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Resupply size (Freedom)</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr"/>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>resupply_kg_freedom</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Printer output</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>kg/sol</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Mars-made material from one running regolith printer fed by a running intake. Pays for room shells, corridors, partitions, shelving, crates and tables.</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>print_kg_per_sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Recycling bonus</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Extra printer output when the base has a plastics recycling hopper (plastic binder).</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>print_recycle_bonus</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U88"/>
+  <dimension ref="A1:U90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8178,15 +8345,156 @@
       </c>
       <c r="U85" s="8" t="n"/>
     </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>regolith_printer</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>Regolith Printer</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="D86" s="13" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E86" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F86" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G86" s="19">
+        <f>E86*F86/24</f>
+        <v/>
+      </c>
+      <c r="H86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T86" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U86" s="8" t="n"/>
+    </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
+          <t>regolith_intake</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Regolith Intake</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>outside</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="E87" s="14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F87" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G87" s="19">
+        <f>E87*F87/24</f>
+        <v/>
+      </c>
+      <c r="H87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S87" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T87" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U87" s="8" t="n"/>
+    </row>
+    <row r="88"/>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
           <t>Example row: grow_tray is 150 kg, uses 0.6 kW for 16 hours a sol (0.4 kW average), grows 0.4 kg of food and uses 0.5 L of water a sol.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="8" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
         <is>
           <t>Positive O2, water and food are made; negative are used. CO2 negative means removed from the air.</t>
         </is>

</xml_diff>

<commit_message>
Fixed-tab build bar with a This room tab, audit room rules, printer-only growth
- Interior build bar: the same tabs in every room, "This room" first with
  only what fits, other tabs greyed out with where each item fits.
- Equipment audit (docs/equipment-audit.md): microscope also in Medical,
  seedling station also in Science, crew chair also in Waste and Life Support.
- Earth resupply switched off (resupply_enabled = 0); Survival starts with
  100 t, Freedom 140 t, and the printer makes 2,500 kg a sol.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Survival starting cargo. Lowered to 80,000 on 22 Oct: resupply landers and the regolith printer now grow the base over time. Freedom starts with more (below). Missions set their own per-landing payloads.</t>
+          <t>Survival starting cargo. Raised to 100,000 on 22 Oct when Earth resupply was switched off: the regolith printer is now how the base grows. Freedom starts with more (below). Missions set their own per-landing payloads.</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>120000</v>
+        <v>140000</v>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Freedom: a generous start and bigger, quicker resupplies.</t>
+          <t>Freedom: a generous start. The regolith printer grows the base from there.</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
@@ -1593,6 +1593,31 @@
       <c r="E36" s="10" t="inlineStr">
         <is>
           <t>print_recycle_bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Earth resupply landers</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>on/off</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1 = resupply landers arrive on launch windows in Survival and Freedom. Switched off (0) on 22 Oct: the regolith printer is the way to grow the base.</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>resupply_enabled</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8510,6 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
-    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Shelves, console, heater and outdoor crate stacking, plus an Odds & Ends pack
- Open shelving takes items on its four upper shelves (with headroom
  checks); its tubs now sit only on the bottom shelf. The planning console
  desk is a surface and the portable heater can go on benches.
- Outdoors, cargo crates stack on the loaded pallet, the workbench and
  each other; removing a surface removes what's on it.
- New Odds & Ends tab: 14 small Blender-modelled items (mug, tablet,
  laptop, books, Earth photo, chess set, zero-g plush, herb pot, desk lamp,
  water bottle, sample jars, toolbox, ration packs, guitar), each with a
  real-world note.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -2213,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U90"/>
+  <dimension ref="A1:U104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8510,6 +8510,7 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
@@ -8521,6 +8522,1042 @@
       <c r="A90" s="8" t="inlineStr">
         <is>
           <t>Positive O2, water and food are made; negative are used. CO2 negative means removed from the air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>crew_mug</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Crew Mug</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91">
+        <f>E91*F91/24</f>
+        <v/>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>0</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0</v>
+      </c>
+      <c r="S91" t="n">
+        <v>0</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0</v>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>crew_tablet</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Crew Tablet</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92">
+        <f>E92*F92/24</f>
+        <v/>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" t="n">
+        <v>0</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0</v>
+      </c>
+      <c r="T92" t="n">
+        <v>0</v>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>crew_laptop</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>2</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93">
+        <f>E93*F93/24</f>
+        <v/>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" t="n">
+        <v>0</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>paper_books</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Paper Books</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94">
+        <f>E94*F94/24</f>
+        <v/>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0</v>
+      </c>
+      <c r="R94" t="n">
+        <v>0</v>
+      </c>
+      <c r="S94" t="n">
+        <v>0</v>
+      </c>
+      <c r="T94" t="n">
+        <v>0</v>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>photo_frame</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Photo Frame</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95">
+        <f>E95*F95/24</f>
+        <v/>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" t="n">
+        <v>0</v>
+      </c>
+      <c r="S95" t="n">
+        <v>0</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0</v>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>chess_set</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Chess Set</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96">
+        <f>E96*F96/24</f>
+        <v/>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0</v>
+      </c>
+      <c r="R96" t="n">
+        <v>0</v>
+      </c>
+      <c r="S96" t="n">
+        <v>0</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0</v>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>zero_g_plush</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Zero-G Plush</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97">
+        <f>E97*F97/24</f>
+        <v/>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" t="n">
+        <v>0</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0</v>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>herb_pot</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Herb Pot</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98">
+        <f>E98*F98/24</f>
+        <v/>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" t="n">
+        <v>0</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0</v>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>desk_lamp</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Desk Lamp</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99">
+        <f>E99*F99/24</f>
+        <v/>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
+        <v>0</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0</v>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>water_bottle</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Water Bottle</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100">
+        <f>E100*F100/24</f>
+        <v/>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" t="n">
+        <v>0</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
+        <v>0</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0</v>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>sample_jars</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Sample Jars</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101">
+        <f>E101*F101/24</f>
+        <v/>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0</v>
+      </c>
+      <c r="R101" t="n">
+        <v>0</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0</v>
+      </c>
+      <c r="T101" t="n">
+        <v>0</v>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>toolbox</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Toolbox</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>6</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102">
+        <f>E102*F102/24</f>
+        <v/>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" t="n">
+        <v>0</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="n">
+        <v>0</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
+      <c r="T102" t="n">
+        <v>0</v>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>ration_packs</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Ration Packs</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103">
+        <f>E103*F103/24</f>
+        <v/>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0</v>
+      </c>
+      <c r="T103" t="n">
+        <v>0</v>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>guitar</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Guitar</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>3</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104">
+        <f>E104*F104/24</f>
+        <v/>
+      </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0</v>
+      </c>
+      <c r="T104" t="n">
+        <v>0</v>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dust storms you can see coming, storm sounds, guitar and plush sounds
- Storms are forecast about 10 hours ahead (alert chime, toast and a
  countdown pill under the sol clock), then cut solar until an all-clear.
  4-8 storms per 100 sols by site, 1.5-2.5 sols long; forecasts are saved.
- New Weather effects setting (off on Low): storm haze, dusty sky, thick
  fog and blowing dust outdoors. Storms happen and are announced either way.
- Synthesised storm roar (outside) and hull buffet (inside), alert and
  all-clear chimes, four guitar strums and three soft plush squeaks; the
  rig's new play action strums the guitar and squeezes the plush.
- Solar telemetry shows the storm's cut. habitat_sim_test no longer
  depends on random storms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1618,6 +1618,31 @@
       <c r="E37" s="10" t="inlineStr">
         <is>
           <t>resupply_enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Storm warning</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>How long before a dust storm the forecast warns you. Real orbiters (MRO) photograph the whole planet every sol, so storms are seen coming.</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>storm_warning_hours</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8535,6 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
-    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
@@ -9830,20 +9854,20 @@
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E10" s="25" t="n">
-        <v>1.2</v>
+        <v>5</v>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>How often a storm hits in Survival. Tests can force one.</t>
+          <t>How often a storm hits in Survival and Freedom (each comes with a forecast warning). Raised on 22 Oct so storms happen in a normal session. Tests can force one.</t>
         </is>
       </c>
     </row>
@@ -9878,18 +9902,22 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C12" s="22" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Shortened on 22 Oct (a sol is about 20 minutes of play). Mission storms set their own length.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Backlog batch 3: building and furniture
New Crew Comforts pack (Blender source in asset_packs/mars_crew_comforts_v1):
a clear work desk, a one-piece galley kitchenette and matching bench units
(the counter, oven and rehydration station are retired from the build bar
but still load from saves), a wall screen and a mini GAR-Y toy. Desks and
wayfinding panels fit in every room.

Interior doors open as you or GAR-Y walk up and close behind you (never
while an outer hatch is open; E pauses them). Partition doors swing away
from whoever opens them, and there is a glass partition door. R switches
partitions to 45° panels. Doors on shared angled walls snap to the 1.5 m
grid.

Wall screens show live habitat status, Mars or Earth; wayfinding panels
show the room, its lights and temperature and an arrow to the nearest
airlock, or a sign you type (F). Both go dark without power.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -2238,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U104"/>
+  <dimension ref="A1:U109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9585,6 +9585,376 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>work_desk_blank</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Work Desk (clear)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>30</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105">
+        <f>E105*F105/24</f>
+        <v/>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" t="n">
+        <v>0</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" t="n">
+        <v>0</v>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>Clear desk for the crew's own laptop, lamp and odds and ends. Placeholder numbers (22 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>galley_kitchenette</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Galley Kitchenette</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>galley</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>200</v>
+      </c>
+      <c r="E106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F106" t="n">
+        <v>3</v>
+      </c>
+      <c r="G106">
+        <f>E106*F106/24</f>
+        <v/>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+      <c r="T106" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>Fridge, sink, hob, oven and rehydration tap in one run; replaces counter, oven and rehydration station. Placeholder numbers (22 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>galley_bench_unit</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Galley Bench Unit</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>galley</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>40</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107">
+        <f>E107*F107/24</f>
+        <v/>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+      <c r="T107" t="n">
+        <v>0</v>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>Matching base cupboards with a clear worktop. Placeholder numbers (22 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>wall_screen</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Wall Screen</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>8</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F108" t="n">
+        <v>12</v>
+      </c>
+      <c r="G108">
+        <f>E108*F108/24</f>
+        <v/>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0</v>
+      </c>
+      <c r="T108" t="n">
+        <v>0</v>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Shows habitat status or a view of Mars or Earth. Placeholder numbers (22 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>mini_gar_y</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Mini GAR-Y</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>odds_and_ends</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109">
+        <f>E109*F109/24</f>
+        <v/>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+      <c r="T109" t="n">
+        <v>0</v>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Odds &amp; ends: personal item, no systems.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Outside camera masts with a 360-degree pan-tilt head
A new outdoor item, the Camera Mast (asset_packs/mars_observation_v1, house
style): a 6 m pole on a ballasted tripod with a pan-tilt camera head, up to
4 per base, delivered in Mission 4. The head physically pans and tilts and
its aim, zoom and auto-sweep are saved with the base.

Mission Control's Cameras button (or E on a mast) opens a live view (game
running, you standing still) through the lens: drag or WASD to aim, wheel
to zoom, Tab or arrows to switch masts, thumbnails of the others, an
Auto-sweep toggle, and a heading/tilt/zoom readout. Wall screens gain a
Camera mode that cycles the masts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -2238,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U109"/>
+  <dimension ref="A1:U110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9955,6 +9955,80 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>camera_mast</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Camera Mast</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>exterior</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>60</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F110" t="n">
+        <v>24</v>
+      </c>
+      <c r="G110">
+        <f>E110*F110/24</f>
+        <v/>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
+        <v>0</v>
+      </c>
+      <c r="S110" t="n">
+        <v>0</v>
+      </c>
+      <c r="T110" t="n">
+        <v>0</v>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>Pan-tilt camera on a 6 m pole. Placeholder numbers (23 Oct).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
One habitat temperature, with a heating coverage rule
Room temperatures are merged into one habitat temperature, like
Subnautica: no per-room targets and no heat flowing between rooms.
Airlocks and the vehicle bay are unheated by design. Placement still
matters through one rule: people, lights and machines warm their own
room; a spot heater warms its room and the rooms next door, up to what
they need (the rest is wasted); the thermal control unit, a ducted heat
pump, reaches every heated room at about three times the heat per kW.
Heated rooms left short are cold spots: a habitat warning, a voiced
alert, and amber on the monitor. The target temperature (21 C) is a new
setting in the balance sheet. Readiness, the monitor, alerts, test
reasons, charts and screens now speak of the habitat's temperature.
Old saves load (their warmest room stands in).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1407,7 +1407,7 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Dangerously cold room</t>
+          <t>Dangerously cold habitat</t>
         </is>
       </c>
       <c r="B29" s="13" t="n">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Crew health falls in rooms below this.</t>
+          <t>Crew health falls when the habitat is below this.</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -1432,215 +1432,240 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Freedom starting cargo</t>
+          <t>Habitat temperature target</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>140000</v>
+        <v>21</v>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Freedom: a generous start. The regolith printer grows the base from there.</t>
+          <t>The heat pump keeps the whole habitat near this. Comfortable is 18 to 24 C. Since 23 Oct the habitat has one temperature (like Subnautica): heaters warm the whole base; airlocks and the vehicle bay are unheated.</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>freedom_cargo_budget_kg</t>
+          <t>habitat_target_c</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Resupply interval (Survival)</t>
+          <t>Freedom starting cargo</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>3</v>
+        <v>140000</v>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>sols</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>A resupply lander arrives this often. Real launch windows are about 26 months apart; the game compresses time.</t>
+          <t>Freedom: a generous start. The regolith printer grows the base from there.</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>resupply_sols_survival</t>
+          <t>freedom_cargo_budget_kg</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Resupply size (Survival)</t>
+          <t>Resupply interval (Survival)</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>15000</v>
+        <v>3</v>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>sols</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Cargo each Survival resupply lander brings.</t>
+          <t>A resupply lander arrives this often. Real launch windows are about 26 months apart; the game compresses time.</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>resupply_kg_survival</t>
+          <t>resupply_sols_survival</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Resupply interval (Freedom)</t>
+          <t>Resupply size (Survival)</t>
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>2</v>
+        <v>15000</v>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>sols</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr"/>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Cargo each Survival resupply lander brings.</t>
+        </is>
+      </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>resupply_sols_freedom</t>
+          <t>resupply_kg_survival</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Resupply size (Freedom)</t>
+          <t>Resupply interval (Freedom)</t>
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>20000</v>
+        <v>2</v>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>sols</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>resupply_kg_freedom</t>
+          <t>resupply_sols_freedom</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Printer output</t>
+          <t>Resupply size (Freedom)</t>
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>kg/sol</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Mars-made material from one running regolith printer fed by a running intake. Pays for room shells, corridors, partitions, shelving, crates and tables.</t>
-        </is>
-      </c>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr"/>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>print_kg_per_sol</t>
+          <t>resupply_kg_freedom</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Recycling bonus</t>
+          <t>Printer output</t>
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>0.25</v>
+        <v>2500</v>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>kg/sol</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Extra printer output when the base has a plastics recycling hopper (plastic binder).</t>
+          <t>Mars-made material from one running regolith printer fed by a running intake. Pays for room shells, corridors, partitions, shelving, crates and tables.</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>print_recycle_bonus</t>
+          <t>print_kg_per_sol</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Earth resupply landers</t>
+          <t>Recycling bonus</t>
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>on/off</t>
+          <t>fraction</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>1 = resupply landers arrive on launch windows in Survival and Freedom. Switched off (0) on 22 Oct: the regolith printer is the way to grow the base.</t>
+          <t>Extra printer output when the base has a plastics recycling hopper (plastic binder).</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>resupply_enabled</t>
+          <t>print_recycle_bonus</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
+          <t>Earth resupply landers</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>on/off</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1 = resupply landers arrive on launch windows in Survival and Freedom. Switched off (0) on 22 Oct: the regolith printer is the way to grow the base.</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>resupply_enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
           <t>Storm warning</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n">
+      <c r="B39" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>hours</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>How long before a dust storm the forecast warns you. Real orbiters (MRO) photograph the whole planet every sol, so storms are seen coming.</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>storm_warning_hours</t>
         </is>
@@ -1699,7 +1724,7 @@
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>Target temperature (C)</t>
+          <t>Target temperature (C) (unused since 23 Oct: one habitat temperature)</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Act 2 core: crew as people, radiation, breaches, breakdowns; Missions 7-10 data
habitat_life.gd: named crew with roles, fitness (exercise in 38% gravity),
wellbeing from six needs, injuries and medical care; one crew radiation
dose with a storm shelter rated in shield points; sections (rooms joined
without a hatch) and one habitat air pressure for breaches, patching and
repressurising; breakdowns repaired with spare parts. Tuning in
data/hazards.json. The mission Test runs events (solar particle event,
injury, breach, blackout) and several futures, with the new checks.
Missions 7-10 in missions.json. Six new house-style models
(mars_living_on_mars_v1). Missions 1-6 unchanged (campaign test passes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -2263,7 +2263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U110"/>
+  <dimension ref="A1:U116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8560,6 +8560,7 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
@@ -10051,6 +10052,450 @@
       <c r="U110" t="inlineStr">
         <is>
           <t>Pan-tilt camera on a 6 m pole. Placeholder numbers (23 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>regolith_shield_block</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Regolith Shield Wall</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>900</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111">
+        <f>E111*F111/24</f>
+        <v/>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
+        <v>0</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0</v>
+      </c>
+      <c r="T111" t="n">
+        <v>0</v>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>Printed regolith blocks: radiation shielding (8 shield points, data/hazards.json). Printable from Mars-made material (23 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>water_wall_panel</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Water Wall</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>260</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112">
+        <f>E112*F112/24</f>
+        <v/>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" t="n">
+        <v>200</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" t="n">
+        <v>0</v>
+      </c>
+      <c r="S112" t="n">
+        <v>0</v>
+      </c>
+      <c r="T112" t="n">
+        <v>0</v>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>200 L water tank used as radiation shielding (10 shield points). Water is hydrogen-rich (23 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>storm_shelter_locker</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Storm Shelter Locker</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>140</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113">
+        <f>E113*F113/24</f>
+        <v/>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+      <c r="T113" t="n">
+        <v>0</v>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>Emergency supplies; its room becomes the storm shelter (Mission 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>hull_patch_kit</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Hull Patch Kit</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>40</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114">
+        <f>E114*F114/24</f>
+        <v/>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="n">
+        <v>0</v>
+      </c>
+      <c r="T114" t="n">
+        <v>0</v>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>Patch plates and sealant: lets the crew patch a breach (Mission 9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t>air_reserve_rack</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Air Reserve Rack</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>life_support</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>380</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115">
+        <f>E115*F115/24</f>
+        <v/>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0</v>
+      </c>
+      <c r="P115" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0</v>
+      </c>
+      <c r="R115" t="n">
+        <v>0</v>
+      </c>
+      <c r="S115" t="n">
+        <v>0</v>
+      </c>
+      <c r="T115" t="n">
+        <v>0</v>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>60 kg of stored air (N2/O2) to refill a vented section (data/hazards.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>spare_parts_rack</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Spare Parts Rack</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>300</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <f>E116*F116/24</f>
+        <v/>
+      </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" t="n">
+        <v>0</v>
+      </c>
+      <c r="S116" t="n">
+        <v>0</v>
+      </c>
+      <c r="T116" t="n">
+        <v>0</v>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>8 spare parts; each repair uses one (Mission 10, data/hazards.json).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch G: Missions 5-10 playtest fixes
The Communications Mast now arrives in Mission 4, and Mission 8 has a
step to set up the Communications room (a station inside, the mast
outside); Contact with Earth needs both. The mission panel shows the whole
current step, how to do it and its progress when collapsed, and the
redundancy step names what still needs a second. Clearer steps in Missions
7-10; Mission 9 tests 4 sols. Mission 5 is a real challenge: a 5 kW
reactor (one allowed), a 7-sol storm and a warmth check. The dossier stays
with a base carried on after the campaign, and thin wall strips can be
removed by aiming at the wall.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -1211,7 +1211,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Like NASA's Kilopower design. Constant day and night.</t>
+          <t>A compact fission reactor, like NASA's Kilopower (1-10 kW). Constant day and night, but it can't carry a whole base alone.</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -8560,7 +8560,6 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
-    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rooms in alphabetical order on the Site plan; Retro Mars Poster
The Site plan's Rooms tab lists rooms alphabetically (1-9 follow it). New
wall decoration: a framed Retro Mars Poster (A home beyond Earth), +1
happiness and one of the crew's personal comforts; in the catalogue, the
balance sheet and resources.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MarsHabitat_Balance.xlsx
+++ b/docs/MarsHabitat_Balance.xlsx
@@ -2263,7 +2263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U116"/>
+  <dimension ref="A1:U117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8560,6 +8560,7 @@
       </c>
       <c r="U87" s="8" t="n"/>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
@@ -9907,19 +9908,19 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="8" t="inlineStr">
-        <is>
-          <t>mini_gar_y</t>
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>retro_mars_poster</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Mini GAR-Y</t>
+          <t>Retro Mars Poster</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>odds_and_ends</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -9976,34 +9977,34 @@
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>Odds &amp; ends: personal item, no systems.</t>
+          <t>Decoration: a framed poster, no systems.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t>camera_mast</t>
+          <t>mini_gar_y</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Camera Mast</t>
+          <t>Mini GAR-Y</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>exterior</t>
+          <t>odds_and_ends</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E110" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G110">
         <f>E110*F110/24</f>
@@ -10050,34 +10051,34 @@
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>Pan-tilt camera on a 6 m pole. Placeholder numbers (23 Oct).</t>
+          <t>Odds &amp; ends: personal item, no systems.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>regolith_shield_block</t>
+          <t>camera_mast</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Regolith Shield Wall</t>
+          <t>Camera Mast</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>exterior</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>900</v>
+        <v>60</v>
       </c>
       <c r="E111" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G111">
         <f>E111*F111/24</f>
@@ -10124,19 +10125,19 @@
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>Printed regolith blocks: radiation shielding (8 shield points, data/hazards.json). Printable from Mars-made material (23 Oct).</t>
+          <t>Pan-tilt camera on a 6 m pole. Placeholder numbers (23 Oct).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t>water_wall_panel</t>
+          <t>regolith_shield_block</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Water Wall</t>
+          <t>Regolith Shield Wall</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -10145,7 +10146,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>260</v>
+        <v>900</v>
       </c>
       <c r="E112" t="n">
         <v>0</v>
@@ -10176,7 +10177,7 @@
         <v>0</v>
       </c>
       <c r="N112" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="O112" t="n">
         <v>0</v>
@@ -10198,28 +10199,28 @@
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>200 L water tank used as radiation shielding (10 shield points). Water is hydrogen-rich (23 Oct).</t>
+          <t>Printed regolith blocks: radiation shielding (8 shield points, data/hazards.json). Printable from Mars-made material (23 Oct).</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t>storm_shelter_locker</t>
+          <t>water_wall_panel</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Storm Shelter Locker</t>
+          <t>Water Wall</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>140</v>
+        <v>260</v>
       </c>
       <c r="E113" t="n">
         <v>0</v>
@@ -10250,7 +10251,7 @@
         <v>0</v>
       </c>
       <c r="N113" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="O113" t="n">
         <v>0</v>
@@ -10272,19 +10273,19 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>Emergency supplies; its room becomes the storm shelter (Mission 7).</t>
+          <t>200 L water tank used as radiation shielding (10 shield points). Water is hydrogen-rich (23 Oct).</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t>hull_patch_kit</t>
+          <t>storm_shelter_locker</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Hull Patch Kit</t>
+          <t>Storm Shelter Locker</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -10293,7 +10294,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="E114" t="n">
         <v>0</v>
@@ -10346,28 +10347,28 @@
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>Patch plates and sealant: lets the crew patch a breach (Mission 9).</t>
+          <t>Emergency supplies; its room becomes the storm shelter (Mission 7).</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>air_reserve_rack</t>
+          <t>hull_patch_kit</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Air Reserve Rack</t>
+          <t>Hull Patch Kit</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>life_support</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>380</v>
+        <v>40</v>
       </c>
       <c r="E115" t="n">
         <v>0</v>
@@ -10420,28 +10421,28 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>60 kg of stored air (N2/O2) to refill a vented section (data/hazards.json).</t>
+          <t>Patch plates and sealant: lets the crew patch a breach (Mission 9).</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>spare_parts_rack</t>
+          <t>air_reserve_rack</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Spare Parts Rack</t>
+          <t>Air Reserve Rack</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>life_support</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>300</v>
+        <v>380</v>
       </c>
       <c r="E116" t="n">
         <v>0</v>
@@ -10493,6 +10494,80 @@
         <v>0</v>
       </c>
       <c r="U116" t="inlineStr">
+        <is>
+          <t>60 kg of stored air (N2/O2) to refill a vented section (data/hazards.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>spare_parts_rack</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Spare Parts Rack</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>300</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <f>E117*F117/24</f>
+        <v/>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0</v>
+      </c>
+      <c r="R117" t="n">
+        <v>0</v>
+      </c>
+      <c r="S117" t="n">
+        <v>0</v>
+      </c>
+      <c r="T117" t="n">
+        <v>0</v>
+      </c>
+      <c r="U117" t="inlineStr">
         <is>
           <t>8 spare parts; each repair uses one (Mission 10, data/hazards.json).</t>
         </is>

</xml_diff>